<commit_message>
sql for Hang lung monthly LMS report booking section
</commit_message>
<xml_diff>
--- a/2026_10/2026_10_02/HangLung_Amoy_Plaza_and_Fashion_Walk_LMS/Hang Lung Monthly LMS Report_Sep 1-30,2026.xlsx
+++ b/2026_10/2026_10_02/HangLung_Amoy_Plaza_and_Fashion_Walk_LMS/Hang Lung Monthly LMS Report_Sep 1-30,2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenalee\work\2026_09\2026_10\2026_10_02\HangLung_Amoy_Plaza_and_Fashion_Walk_LMS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DD6443FD-72F5-44C0-853C-90F64554A96B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0AB8DE2B-A759-4776-A05A-AD724299A12B}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19200" windowHeight="6285" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="68">
   <si>
     <t>Advertiser :</t>
   </si>
@@ -219,6 +219,15 @@
   </si>
   <si>
     <t>HOKA</t>
+  </si>
+  <si>
+    <t>牛気</t>
+  </si>
+  <si>
+    <t>阿城鵝肉</t>
+  </si>
+  <si>
+    <t>鮨政</t>
   </si>
 </sst>
 </file>
@@ -890,7 +899,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="62">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -1044,6 +1053,7 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="36" borderId="10" xfId="42" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="44">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1095,9 +1105,9 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFFF99FF"/>
       <color rgb="FF0000FF"/>
       <color rgb="FFFF66CC"/>
-      <color rgb="FFFF99FF"/>
     </mruColors>
   </colors>
   <extLst>
@@ -2057,12 +2067,24 @@
       <c r="H8" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="I8" s="16"/>
-      <c r="J8" s="18"/>
-      <c r="K8" s="18"/>
-      <c r="L8" s="18"/>
-      <c r="M8" s="18"/>
-      <c r="N8" s="18"/>
+      <c r="I8" s="16">
+        <v>914</v>
+      </c>
+      <c r="J8" s="18">
+        <v>5</v>
+      </c>
+      <c r="K8" s="18">
+        <v>622</v>
+      </c>
+      <c r="L8" s="18">
+        <v>18</v>
+      </c>
+      <c r="M8" s="18">
+        <v>20</v>
+      </c>
+      <c r="N8" s="18">
+        <v>1562</v>
+      </c>
       <c r="O8" s="6"/>
     </row>
     <row r="9" spans="1:25" s="1" customFormat="1" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2088,12 +2110,24 @@
       <c r="H9" s="17" t="s">
         <v>22</v>
       </c>
-      <c r="I9" s="18"/>
-      <c r="J9" s="18"/>
-      <c r="K9" s="18"/>
-      <c r="L9" s="18"/>
-      <c r="M9" s="18"/>
-      <c r="N9" s="18"/>
+      <c r="I9" s="18">
+        <v>2377</v>
+      </c>
+      <c r="J9" s="18">
+        <v>12</v>
+      </c>
+      <c r="K9" s="18">
+        <v>4083</v>
+      </c>
+      <c r="L9" s="18">
+        <v>4</v>
+      </c>
+      <c r="M9" s="18">
+        <v>5</v>
+      </c>
+      <c r="N9" s="61">
+        <v>2317</v>
+      </c>
       <c r="O9" s="6"/>
     </row>
     <row r="10" spans="1:25" ht="33" customHeight="1" x14ac:dyDescent="0.25">
@@ -2127,7 +2161,9 @@
       <c r="B12" s="36" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="33"/>
+      <c r="C12" s="33" t="s">
+        <v>46</v>
+      </c>
       <c r="D12" s="33" t="s">
         <v>55</v>
       </c>
@@ -2151,7 +2187,9 @@
       <c r="B13" s="36" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="33"/>
+      <c r="C13" s="33" t="s">
+        <v>65</v>
+      </c>
       <c r="D13" s="33" t="s">
         <v>56</v>
       </c>
@@ -2176,7 +2214,9 @@
       <c r="B14" s="36" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="33"/>
+      <c r="C14" s="33" t="s">
+        <v>66</v>
+      </c>
       <c r="D14" s="33" t="s">
         <v>57</v>
       </c>
@@ -2266,7 +2306,9 @@
       <c r="B19" s="36" t="s">
         <v>50</v>
       </c>
-      <c r="C19" s="33"/>
+      <c r="C19" s="33" t="s">
+        <v>51</v>
+      </c>
       <c r="D19" s="33" t="s">
         <v>60</v>
       </c>
@@ -2279,7 +2321,9 @@
       <c r="B20" s="36" t="s">
         <v>51</v>
       </c>
-      <c r="C20" s="33"/>
+      <c r="C20" s="33" t="s">
+        <v>50</v>
+      </c>
       <c r="D20" s="33" t="s">
         <v>61</v>
       </c>
@@ -2294,7 +2338,9 @@
       <c r="B21" s="36" t="s">
         <v>52</v>
       </c>
-      <c r="C21" s="33"/>
+      <c r="C21" s="33" t="s">
+        <v>53</v>
+      </c>
       <c r="D21" s="33" t="s">
         <v>62</v>
       </c>
@@ -2320,7 +2366,9 @@
       <c r="B22" s="36" t="s">
         <v>53</v>
       </c>
-      <c r="C22" s="33"/>
+      <c r="C22" s="33" t="s">
+        <v>54</v>
+      </c>
       <c r="D22" s="33" t="s">
         <v>63</v>
       </c>
@@ -2332,7 +2380,9 @@
       <c r="B23" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="C23" s="33"/>
+      <c r="C23" s="33" t="s">
+        <v>67</v>
+      </c>
       <c r="D23" s="33" t="s">
         <v>64</v>
       </c>

</xml_diff>